<commit_message>
vault backup: 2026-09-18 23:02:05
</commit_message>
<xml_diff>
--- a/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
+++ b/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
@@ -1146,7 +1146,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-09-19 23:28:28
</commit_message>
<xml_diff>
--- a/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
+++ b/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
@@ -12,6 +12,7 @@
     <sheet name="주간조정" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="계좌목록" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="정기지출분류" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="공휴일" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2003,4 +2004,122 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>일자</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>이름</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>(안내) 해마다 설날·추석·임시공휴일 등을 여기에 추가하세요. 일자·요일이 결과물에서 붉은 글자로 표시됩니다.</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>추석 연휴</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>추석</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>추석 연휴</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>개천절</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>개천절 대체공휴일</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>한글날</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>46381</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>성탄절</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>46388</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>신정</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-09-20 00:09:06
</commit_message>
<xml_diff>
--- a/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
+++ b/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
@@ -1130,7 +1130,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1385,7 +1385,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1538,7 +1538,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1572,7 +1572,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1606,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1640,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1759,7 +1759,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1810,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1827,7 +1827,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1878,7 +1878,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1895,7 +1895,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1929,7 +1929,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1963,7 +1963,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1997,7 +1997,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -2037,7 +2037,6 @@
           <t>(안내) 해마다 설날·추석·임시공휴일 등을 여기에 추가하세요. 일자·요일이 결과물에서 붉은 글자로 표시됩니다.</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">

</xml_diff>

<commit_message>
vault backup: 2026-09-20 00:19:17
</commit_message>
<xml_diff>
--- a/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
+++ b/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
@@ -1130,7 +1130,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1385,7 +1385,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1606,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1759,7 +1759,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1827,7 +1827,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1878,7 +1878,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1929,7 +1929,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1997,7 +1997,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-09-20 00:29:27
</commit_message>
<xml_diff>
--- a/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
+++ b/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
@@ -1130,7 +1130,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-09-20 00:39:38
</commit_message>
<xml_diff>
--- a/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
+++ b/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
@@ -1147,7 +1147,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1606,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1759,7 +1759,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1827,7 +1827,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-09-20 00:59:39
</commit_message>
<xml_diff>
--- a/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
+++ b/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
@@ -1130,7 +1130,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1538,7 +1538,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1606,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1640,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1759,7 +1759,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1827,7 +1827,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1895,7 +1895,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1963,7 +1963,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-09-20 01:30:00
</commit_message>
<xml_diff>
--- a/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
+++ b/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
@@ -1130,7 +1130,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1385,7 +1385,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1538,7 +1538,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1606,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1640,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1759,7 +1759,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1827,7 +1827,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1878,7 +1878,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1895,7 +1895,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1929,7 +1929,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1963,7 +1963,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>제외</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>
@@ -1997,7 +1997,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-09-20 01:40:10
</commit_message>
<xml_diff>
--- a/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
+++ b/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
@@ -1130,7 +1130,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1385,7 +1385,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1538,7 +1538,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1606,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1640,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1759,7 +1759,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1827,7 +1827,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1878,7 +1878,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1895,7 +1895,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1929,7 +1929,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1963,7 +1963,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>제외</t>
         </is>
       </c>
     </row>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1997,7 +1997,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-09-20 01:50:21
</commit_message>
<xml_diff>
--- a/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
+++ b/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
@@ -1232,7 +1232,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>변동</t>
+          <t>정기</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>정기</t>
+          <t>변동</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-09-21 20:20:34
</commit_message>
<xml_diff>
--- a/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
+++ b/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
@@ -1090,7 +1090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1996,6 +1996,74 @@
         </is>
       </c>
       <c r="C54" t="inlineStr">
+        <is>
+          <t>정기</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>국민네이버 apha</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>광고비</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>변동</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>주식회사에이팜건강</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>자계자 이체</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>변동</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>국민네이버 에이팜건</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>광고비</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>변동</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>국민주에이팜건강</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>자계자 이체</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
         <is>
           <t>정기</t>
         </is>

</xml_diff>

<commit_message>
vault backup: 2026-10-05 00:14:29
</commit_message>
<xml_diff>
--- a/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
+++ b/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/04_기준파일/에이팜건강_자금계획_기준파일.xlsx
@@ -1090,7 +1090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2064,6 +2064,19 @@
         </is>
       </c>
       <c r="C58" t="inlineStr">
+        <is>
+          <t>정기</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>가스</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr">
         <is>
           <t>정기</t>
         </is>

</xml_diff>